<commit_message>
docs & telemetry: complete code cleanup, comprehensive markdown documentation and protocol specification
</commit_message>
<xml_diff>
--- a/docs/펌웨어 테스트.xlsx
+++ b/docs/펌웨어 테스트.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\stm32\COSMOKE_H563\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C336F14F-9170-4958-AC53-C28153C1ADB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF362857-7B7E-4304-8786-DDBB3FA11FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="354">
   <si>
     <t>COSMOKE H563 펌웨어 성능 시험 기록표</t>
   </si>
@@ -91,9 +91,6 @@
     <t>펌웨어 성능 시험 계획</t>
   </si>
   <si>
-    <t>목표값은 프로젝트 요구사항에 맞게 승인 후 수정하십시오. Test Log에 동일한 ID로 실제 결과를 기록합니다.</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -166,18 +163,9 @@
     <t>A-02</t>
   </si>
   <si>
-    <t>gain 오차</t>
-  </si>
-  <si>
-    <t>100% span 오차</t>
-  </si>
-  <si>
     <t>정밀 전압·전류원</t>
   </si>
   <si>
-    <t>보정 전/후 비교</t>
-  </si>
-  <si>
     <t>A-03</t>
   </si>
   <si>
@@ -382,19 +370,10 @@
     <t>4b7b1d3 (pre-gain)</t>
   </si>
   <si>
-    <t>CH1·CH2 gain</t>
-  </si>
-  <si>
     <t>100% span 최대 오차</t>
   </si>
   <si>
-    <t>11 V / 5 A; CH1+CH2; user-induced input interruption excluded</t>
-  </si>
-  <si>
     <t>현장 검증 이관</t>
-  </si>
-  <si>
-    <t>벤치 합격 판정에서는 제외. 보정 전 데이터와 SCALE_TRIM 적용 이력은 보존하며 실제 운용 환경에서 검증.</t>
   </si>
   <si>
     <t>logs/cosmoke_capture_20260820_094031_980220.csv</t>
@@ -1178,6 +1157,208 @@
     </r>
     <phoneticPr fontId="21" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">11V/5A </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">인 가 시 추가적인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">OFFSET </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이때의 파워 서플라이 출력은 멀티미터로 2차확인 완료</t>
+    </r>
+    <phoneticPr fontId="21" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>전</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>비교</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <phoneticPr fontId="21" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>영점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>오차</t>
+    </r>
+    <phoneticPr fontId="21" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">15V/5A </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>입력시 오차</t>
+    </r>
+    <phoneticPr fontId="21" type="noConversion"/>
+  </si>
+  <si>
+    <t>11 V / 5 A; CH1+CH2; user-induced input interruption excluded</t>
+    <phoneticPr fontId="21" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CH1·CH2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>영점</t>
+    </r>
+    <phoneticPr fontId="21" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1190,7 +1371,7 @@
     <numFmt numFmtId="179" formatCode="0.000000"/>
     <numFmt numFmtId="180" formatCode="0.0"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1346,6 +1527,41 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F2937"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
+      <name val="Aptos"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2937"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="17">
     <fill>
@@ -1497,7 +1713,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1641,6 +1857,20 @@
     <xf numFmtId="180" fontId="7" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1653,11 +1883,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1667,9 +1896,6 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1677,17 +1903,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2249,34 +2470,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1">
-      <c r="A1" s="71" t="s">
-        <v>354</v>
-      </c>
-      <c r="B1" s="55" t="s">
+      <c r="A1" s="60" t="s">
+        <v>347</v>
+      </c>
+      <c r="B1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="55" t="s">
+      <c r="C1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="55" t="s">
+      <c r="E1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="55" t="s">
+      <c r="F1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="55" t="s">
+      <c r="G1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="55" t="s">
+      <c r="H1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="55" t="s">
+      <c r="I1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="55" t="s">
+      <c r="J1" s="61" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2293,18 +2514,18 @@
       <c r="J2" s="23"/>
     </row>
     <row r="3" spans="1:10" ht="28" hidden="1" customHeight="1">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="23"/>
@@ -2319,34 +2540,34 @@
       <c r="J4" s="23"/>
     </row>
     <row r="5" spans="1:10" ht="22" customHeight="1">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="57" t="s">
+      <c r="C5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="57" t="s">
+      <c r="D5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="57" t="s">
+      <c r="E5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="57" t="s">
+      <c r="F5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="57" t="s">
+      <c r="G5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="57" t="s">
+      <c r="H5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="I5" s="57" t="s">
+      <c r="I5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="J5" s="57" t="s">
+      <c r="J5" s="63" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2359,25 +2580,25 @@
         <v>9</v>
       </c>
       <c r="C6" s="23"/>
-      <c r="D6" s="58" t="s">
+      <c r="D6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="58" t="s">
+      <c r="E6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="58" t="s">
+      <c r="F6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="58" t="s">
+      <c r="G6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="58" t="s">
+      <c r="H6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="58" t="s">
+      <c r="I6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="58" t="s">
+      <c r="J6" s="64" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2753,64 +2974,64 @@
       <c r="J30" s="23"/>
     </row>
     <row r="31" spans="1:10" ht="14" customHeight="1">
-      <c r="A31" s="72"/>
-      <c r="B31" s="72"/>
-      <c r="C31" s="72"/>
-      <c r="D31" s="72"/>
-      <c r="E31" s="72"/>
-      <c r="F31" s="72"/>
-      <c r="G31" s="72"/>
-      <c r="H31" s="72"/>
-      <c r="I31" s="72"/>
-      <c r="J31" s="72"/>
+      <c r="A31" s="23"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
     </row>
     <row r="32" spans="1:10" ht="22" customHeight="1">
-      <c r="A32" s="72"/>
-      <c r="B32" s="72"/>
-      <c r="C32" s="72"/>
-      <c r="D32" s="72"/>
-      <c r="E32" s="72"/>
-      <c r="F32" s="72"/>
-      <c r="G32" s="72"/>
-      <c r="H32" s="72"/>
-      <c r="I32" s="72"/>
-      <c r="J32" s="72"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
     </row>
     <row r="33" spans="1:10" ht="34" customHeight="1">
-      <c r="A33" s="72"/>
-      <c r="B33" s="72"/>
-      <c r="C33" s="72"/>
-      <c r="D33" s="72"/>
-      <c r="E33" s="72"/>
-      <c r="F33" s="72"/>
-      <c r="G33" s="72"/>
-      <c r="H33" s="72"/>
-      <c r="I33" s="72"/>
-      <c r="J33" s="72"/>
+      <c r="A33" s="23"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23"/>
     </row>
     <row r="34" spans="1:10" ht="26" customHeight="1">
-      <c r="A34" s="72"/>
-      <c r="B34" s="72"/>
-      <c r="C34" s="72"/>
-      <c r="D34" s="72"/>
-      <c r="E34" s="72"/>
-      <c r="F34" s="72"/>
-      <c r="G34" s="72"/>
-      <c r="H34" s="72"/>
-      <c r="I34" s="72"/>
-      <c r="J34" s="72"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
     </row>
     <row r="35" spans="1:10" ht="26" customHeight="1">
-      <c r="A35" s="73"/>
-      <c r="B35" s="73"/>
-      <c r="C35" s="73"/>
-      <c r="D35" s="73"/>
-      <c r="E35" s="73"/>
-      <c r="F35" s="73"/>
-      <c r="G35" s="73"/>
-      <c r="H35" s="73"/>
-      <c r="I35" s="73"/>
-      <c r="J35" s="73"/>
+      <c r="A35" s="55"/>
+      <c r="B35" s="55"/>
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
+      <c r="E35" s="55"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="55"/>
+      <c r="H35" s="55"/>
+      <c r="I35" s="55"/>
+      <c r="J35" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2853,34 +3074,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="59" t="s">
+      <c r="D1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="59" t="s">
+      <c r="E1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="59" t="s">
+      <c r="F1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="59" t="s">
+      <c r="G1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="59" t="s">
+      <c r="H1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="59" t="s">
+      <c r="I1" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="59" t="s">
+      <c r="J1" s="58" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2897,18 +3118,16 @@
       <c r="J2" s="23"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="60" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
+      <c r="A3" s="65"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="23"/>
@@ -2924,258 +3143,258 @@
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1">
       <c r="A5" s="36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" s="36" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="36" t="s">
+      <c r="E5" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="F5" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="36" t="s">
+      <c r="G5" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="36" t="s">
+      <c r="H5" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="36" t="s">
+      <c r="I5" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="J5" s="36" t="s">
         <v>25</v>
-      </c>
-      <c r="J5" s="36" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="34" customHeight="1">
       <c r="A6" s="40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="37" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="E6" s="37" t="s">
         <v>29</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>30</v>
       </c>
       <c r="F6" s="38">
         <v>3</v>
       </c>
       <c r="G6" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="I6" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="I6" s="37" t="s">
+      <c r="J6" s="37" t="s">
         <v>33</v>
-      </c>
-      <c r="J6" s="37" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="34" customHeight="1">
       <c r="A7" s="40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="37" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="E7" s="37" t="s">
         <v>37</v>
-      </c>
-      <c r="E7" s="37" t="s">
-        <v>38</v>
       </c>
       <c r="F7" s="38">
         <v>0.2</v>
       </c>
       <c r="G7" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H7" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="J7" s="37" t="s">
         <v>39</v>
-      </c>
-      <c r="I7" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="J7" s="37" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="34" customHeight="1">
       <c r="A8" s="40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="37" t="s">
-        <v>42</v>
+      <c r="C8" s="57" t="s">
+        <v>350</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>43</v>
+        <v>351</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F8" s="38">
         <v>0.5</v>
       </c>
       <c r="G8" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I8" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="37" t="s">
-        <v>45</v>
+        <v>32</v>
+      </c>
+      <c r="J8" s="56" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="34" customHeight="1">
       <c r="A9" s="40" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B9" s="37" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F9" s="38">
         <v>1</v>
       </c>
       <c r="G9" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I9" s="37" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="34" customHeight="1">
       <c r="A10" s="40" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B10" s="37" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F10" s="38">
         <v>50</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="34" customHeight="1">
       <c r="A11" s="40" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B11" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F11" s="38">
         <v>1980</v>
       </c>
       <c r="G11" s="37" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H11" s="37" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I11" s="37" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J11" s="37" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="34" customHeight="1">
       <c r="A12" s="40" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B12" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F12" s="38">
         <v>0</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="34" customHeight="1">
@@ -3192,98 +3411,98 @@
     </row>
     <row r="14" spans="1:10" ht="34" customHeight="1">
       <c r="A14" s="40" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B14" s="37" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F14" s="38">
         <v>100</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="34" customHeight="1">
       <c r="A15" s="40" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B15" s="37" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F15" s="38">
         <v>0.1</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H15" s="37" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="I15" s="37" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J15" s="37" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="34" customHeight="1">
       <c r="A16" s="40" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B16" s="37" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F16" s="38">
         <v>25</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -3346,93 +3565,93 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="3" max="3" width="22" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="17" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="9" customWidth="1"/>
+    <col min="9" max="9" width="9" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="12" width="12" customWidth="1"/>
     <col min="13" max="14" width="13" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
     <col min="16" max="16" width="30" customWidth="1"/>
-    <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="17" max="17" width="11" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="17" customWidth="1"/>
-    <col min="19" max="19" width="12" customWidth="1"/>
+    <col min="19" max="19" width="12" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="38" customWidth="1"/>
     <col min="21" max="21" width="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="30" customHeight="1">
-      <c r="A1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="B1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="E1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="G1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="H1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="I1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="J1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="K1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="L1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="M1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="N1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="O1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="P1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="R1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="S1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="T1" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="U1" s="59" t="s">
-        <v>89</v>
+      <c r="A1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="I1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="K1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="L1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="M1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="N1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="O1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="P1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="R1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="S1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="T1" s="58" t="s">
+        <v>85</v>
+      </c>
+      <c r="U1" s="58" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -3459,29 +3678,29 @@
       <c r="U2" s="41"/>
     </row>
     <row r="3" spans="1:21">
-      <c r="A3" s="61" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="61"/>
-      <c r="M3" s="61"/>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="61"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="61"/>
-      <c r="U3" s="61"/>
+      <c r="A3" s="59" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+      <c r="R3" s="59"/>
+      <c r="S3" s="59"/>
+      <c r="T3" s="59"/>
+      <c r="U3" s="59"/>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" s="41"/>
@@ -3508,96 +3727,96 @@
     </row>
     <row r="5" spans="1:21" ht="34" customHeight="1">
       <c r="A5" s="42" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D5" s="42" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="42" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="G5" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="42" t="s">
-        <v>21</v>
-      </c>
       <c r="H5" s="42" t="s">
+        <v>89</v>
+      </c>
+      <c r="I5" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="K5" s="42" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="N5" s="42" t="s">
+        <v>92</v>
+      </c>
+      <c r="O5" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="I5" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" s="42" t="s">
+      <c r="P5" s="42" t="s">
         <v>94</v>
       </c>
-      <c r="K5" s="42" t="s">
-        <v>61</v>
-      </c>
-      <c r="L5" s="42" t="s">
-        <v>31</v>
-      </c>
-      <c r="M5" s="42" t="s">
+      <c r="Q5" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="N5" s="42" t="s">
+      <c r="R5" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="O5" s="42" t="s">
+      <c r="S5" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="P5" s="42" t="s">
+      <c r="T5" s="42" t="s">
+        <v>25</v>
+      </c>
+      <c r="U5" s="42" t="s">
         <v>98</v>
-      </c>
-      <c r="Q5" s="42" t="s">
-        <v>99</v>
-      </c>
-      <c r="R5" s="42" t="s">
-        <v>100</v>
-      </c>
-      <c r="S5" s="42" t="s">
-        <v>101</v>
-      </c>
-      <c r="T5" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="U5" s="42" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="42" customHeight="1">
       <c r="A6" s="47" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="44">
         <v>46254</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="43" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="43" t="s">
+      <c r="G6" s="43" t="s">
         <v>29</v>
-      </c>
-      <c r="G6" s="43" t="s">
-        <v>30</v>
       </c>
       <c r="H6" s="48">
         <v>3</v>
       </c>
       <c r="I6" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J6" s="49">
         <v>2.3119999999999998</v>
@@ -3612,52 +3831,52 @@
         <v>1</v>
       </c>
       <c r="P6" s="45" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="Q6" s="50" t="str">
         <f>IF(OR(H6="",I6="",J6=""),"INPUT",IF(I6="최대",IF(J6&lt;=H6,"PASS","FAIL"),IF(I6="최소",IF(J6&gt;=H6,"PASS","FAIL"),IF(I6="일치",IF(J6=H6,"PASS","FAIL"),"CHECK"))))</f>
         <v>PASS</v>
       </c>
       <c r="R6" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S6" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T6" s="45" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="U6" s="45" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="42" customHeight="1">
       <c r="A7" s="47" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="44">
         <v>46254</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D7" s="43" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F7" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G7" s="43" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H7" s="48">
         <v>0.2</v>
       </c>
       <c r="I7" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J7" s="49">
         <v>4.1553E-2</v>
@@ -3678,52 +3897,52 @@
         <v>3001</v>
       </c>
       <c r="P7" s="45" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="Q7" s="50" t="str">
         <f>IF(OR(H7="",I7="",J7=""),"INPUT",IF(I7="최대",IF(J7&lt;=H7,"PASS","FAIL"),IF(I7="최소",IF(J7&gt;=H7,"PASS","FAIL"),IF(I7="일치",IF(J7=H7,"PASS","FAIL"),"CHECK"))))</f>
         <v>PASS</v>
       </c>
       <c r="R7" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S7" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T7" s="45" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="U7" s="45" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="42" customHeight="1">
       <c r="A8" s="47" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="44">
         <v>46254</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>114</v>
+        <v>353</v>
       </c>
       <c r="F8" s="43" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="G8" s="43" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H8" s="48">
         <v>0.5</v>
       </c>
       <c r="I8" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J8" s="49">
         <v>10.4435</v>
@@ -3744,52 +3963,52 @@
         <v>16577</v>
       </c>
       <c r="P8" s="45" t="s">
-        <v>116</v>
+        <v>352</v>
       </c>
       <c r="Q8" s="50" t="str">
         <f>"FIELD"</f>
         <v>FIELD</v>
       </c>
       <c r="R8" s="51" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="S8" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T8" s="45" t="s">
-        <v>118</v>
+        <v>348</v>
       </c>
       <c r="U8" s="45" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="42" customHeight="1">
       <c r="A9" s="47" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B9" s="44">
         <v>46254</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D9" s="43" t="s">
         <v>11</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F9" s="43" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G9" s="43" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H9" s="48">
         <v>1</v>
       </c>
       <c r="I9" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J9" s="49">
         <v>0.28029999999999999</v>
@@ -3810,52 +4029,52 @@
         <v>3</v>
       </c>
       <c r="P9" s="45" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="Q9" s="50" t="str">
         <f>IF(OR(H9="",I9="",J9=""),"INPUT",IF(I9="최대",IF(J9&lt;=H9,"PASS","FAIL"),IF(I9="최소",IF(J9&gt;=H9,"PASS","FAIL"),IF(I9="일치",IF(J9=H9,"PASS","FAIL"),"CHECK"))))</f>
         <v>PASS</v>
       </c>
       <c r="R9" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S9" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T9" s="45" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="U9" s="45" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="42" customHeight="1">
       <c r="A10" s="47" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B10" s="44">
         <v>46254</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="43" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="F10" s="43" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G10" s="43" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H10" s="48">
         <v>50</v>
       </c>
       <c r="I10" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J10" s="49">
         <v>18.206</v>
@@ -3876,52 +4095,52 @@
         <v>3001</v>
       </c>
       <c r="P10" s="45" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="Q10" s="50" t="str">
         <f>IF(OR(H10="",I10="",J10=""),"INPUT",IF(I10="최대",IF(J10&lt;=H10,"PASS","FAIL"),IF(I10="최소",IF(J10&gt;=H10,"PASS","FAIL"),IF(I10="일치",IF(J10=H10,"PASS","FAIL"),"CHECK"))))</f>
         <v>PASS</v>
       </c>
       <c r="R10" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S10" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T10" s="45" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="U10" s="45" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="42" customHeight="1">
       <c r="A11" s="47" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B11" s="44">
         <v>46254</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D11" s="43" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F11" s="43" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G11" s="43" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H11" s="48">
         <v>1980</v>
       </c>
       <c r="I11" s="46" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J11" s="49">
         <v>1999.931</v>
@@ -3936,52 +4155,52 @@
         <v>16621</v>
       </c>
       <c r="P11" s="45" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="Q11" s="50" t="str">
         <f>IF(J11&gt;=H11,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="R11" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S11" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T11" s="45" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="U11" s="45" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="42" customHeight="1">
       <c r="A12" s="47" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B12" s="44">
         <v>46254</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D12" s="43" t="s">
         <v>13</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F12" s="43" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G12" s="43" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H12" s="48">
         <v>0</v>
       </c>
       <c r="I12" s="46" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J12" s="49">
         <v>0</v>
@@ -4002,26 +4221,26 @@
         <v>16621</v>
       </c>
       <c r="P12" s="45" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="Q12" s="50" t="str">
         <f>IF(J12=0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="R12" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S12" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T12" s="45" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="U12" s="45" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" ht="42" customHeight="1">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="42" hidden="1" customHeight="1">
       <c r="A13" s="47"/>
       <c r="B13" s="44"/>
       <c r="C13" s="45"/>
@@ -4046,31 +4265,31 @@
     </row>
     <row r="14" spans="1:21" ht="42" customHeight="1">
       <c r="A14" s="47" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B14" s="44">
         <v>46254</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>14</v>
       </c>
       <c r="E14" s="43" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F14" s="43" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G14" s="43" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H14" s="48">
         <v>100</v>
       </c>
       <c r="I14" s="46" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="J14" s="49">
         <v>99.998999999999995</v>
@@ -4091,52 +4310,52 @@
         <v>16620</v>
       </c>
       <c r="P14" s="45" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="Q14" s="50" t="str">
         <f>IF(AND(J14&gt;=95,J14&lt;=105),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="R14" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S14" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T14" s="45" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="U14" s="45" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:21" ht="42" customHeight="1">
       <c r="A15" s="47" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B15" s="44">
         <v>46254</v>
       </c>
       <c r="C15" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>14</v>
       </c>
       <c r="E15" s="43" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F15" s="43" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G15" s="43" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H15" s="48">
         <v>0.1</v>
       </c>
       <c r="I15" s="46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J15" s="49">
         <v>0</v>
@@ -4157,52 +4376,52 @@
         <v>16620</v>
       </c>
       <c r="P15" s="45" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="Q15" s="50" t="str">
         <f>IF(J15&lt;=H15,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="R15" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S15" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T15" s="45" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="U15" s="45" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="42" customHeight="1">
       <c r="A16" s="47" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B16" s="44">
         <v>46254</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>15</v>
       </c>
       <c r="E16" s="43" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F16" s="43" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G16" s="43" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H16" s="48">
         <v>25</v>
       </c>
       <c r="I16" s="46" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J16" s="49">
         <v>27.7</v>
@@ -4221,26 +4440,26 @@
         <v>16621</v>
       </c>
       <c r="P16" s="45" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="Q16" s="50" t="str">
         <f>IF(J16&gt;=H16,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="R16" s="51" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="S16" s="45" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="T16" s="45" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="U16" s="45" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" hidden="1">
       <c r="A17" s="1"/>
       <c r="B17" s="5"/>
       <c r="C17" s="4"/>
@@ -4263,7 +4482,7 @@
       <c r="T17" s="4"/>
       <c r="U17" s="4"/>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:21" hidden="1">
       <c r="A18" s="1"/>
       <c r="B18" s="5"/>
       <c r="C18" s="4"/>
@@ -4286,7 +4505,7 @@
       <c r="T18" s="4"/>
       <c r="U18" s="4"/>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:21" hidden="1">
       <c r="A19" s="1"/>
       <c r="B19" s="5"/>
       <c r="C19" s="4"/>
@@ -4309,7 +4528,7 @@
       <c r="T19" s="4"/>
       <c r="U19" s="4"/>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:21" hidden="1">
       <c r="A20" s="1"/>
       <c r="B20" s="5"/>
       <c r="C20" s="4"/>
@@ -4332,6 +4551,7 @@
       <c r="T20" s="4"/>
       <c r="U20" s="4"/>
     </row>
+    <row r="21" spans="1:21" hidden="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:U1"/>
@@ -4374,29 +4594,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="E1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="F1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="G1" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="H1" s="59" t="s">
-        <v>135</v>
+      <c r="A1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="C1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="D1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" s="58" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4410,16 +4630,16 @@
       <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
+      <c r="A3" s="65" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="23"/>
@@ -4433,33 +4653,33 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
       <c r="A5" s="36" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="H5" s="36" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="32" customHeight="1">
       <c r="A6" s="39" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B6" s="52">
         <v>0.05</v>
@@ -4474,18 +4694,18 @@
         <v>0.02</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="G6" s="37" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="32" customHeight="1">
       <c r="A7" s="39" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B7" s="52">
         <v>10</v>
@@ -4500,18 +4720,18 @@
         <v>10</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G7" s="37" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="32" customHeight="1">
       <c r="A8" s="39" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="B8" s="52">
         <v>100</v>
@@ -4526,18 +4746,18 @@
         <v>100</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G8" s="37" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="32" customHeight="1">
       <c r="A9" s="39" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B9" s="52">
         <v>256</v>
@@ -4552,18 +4772,18 @@
         <v>128</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="G9" s="37" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="H9" s="37" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="32" customHeight="1">
       <c r="A10" s="39" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="B10" s="52">
         <v>500</v>
@@ -4578,18 +4798,18 @@
         <v>500</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="32" customHeight="1">
       <c r="A11" s="39" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B11" s="52">
         <v>16</v>
@@ -4604,18 +4824,18 @@
         <v>16</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G11" s="37" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="H11" s="37" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="32" customHeight="1">
       <c r="A12" s="39" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B12" s="52">
         <v>2000</v>
@@ -4630,13 +4850,13 @@
         <v>2000</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -4665,381 +4885,381 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="62" t="s">
-        <v>167</v>
-      </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
+      <c r="A1" s="67" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1">
-      <c r="A3" s="63" t="s">
-        <v>168</v>
-      </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
+      <c r="A3" s="68" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
     </row>
     <row r="5" spans="1:8" ht="22" customHeight="1">
-      <c r="A5" s="64" t="s">
-        <v>169</v>
-      </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="64"/>
-      <c r="F5" s="64"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="64"/>
+      <c r="A5" s="69" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="69"/>
+      <c r="C5" s="69"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
     </row>
     <row r="6" spans="1:8" ht="28" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="B6" s="65" t="s">
-        <v>171</v>
-      </c>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
+        <v>163</v>
+      </c>
+      <c r="B6" s="66" t="s">
+        <v>164</v>
+      </c>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
     </row>
     <row r="7" spans="1:8" ht="28" customHeight="1">
       <c r="A7" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B7" s="65" t="s">
-        <v>173</v>
-      </c>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="65"/>
+        <v>165</v>
+      </c>
+      <c r="B7" s="66" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
     </row>
     <row r="8" spans="1:8" ht="28" customHeight="1">
       <c r="A8" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="B8" s="65" t="s">
-        <v>175</v>
-      </c>
-      <c r="C8" s="65"/>
-      <c r="D8" s="65"/>
-      <c r="E8" s="65"/>
-      <c r="F8" s="65"/>
-      <c r="G8" s="65"/>
-      <c r="H8" s="65"/>
+        <v>167</v>
+      </c>
+      <c r="B8" s="66" t="s">
+        <v>168</v>
+      </c>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="G8" s="66"/>
+      <c r="H8" s="66"/>
     </row>
     <row r="9" spans="1:8" ht="28" customHeight="1">
       <c r="A9" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B9" s="65" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
+        <v>169</v>
+      </c>
+      <c r="B9" s="66" t="s">
+        <v>170</v>
+      </c>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1">
       <c r="A11" s="33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="58" customHeight="1">
       <c r="A12" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="37" t="s">
-        <v>28</v>
-      </c>
       <c r="C12" s="37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="F12" s="53" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="58" customHeight="1">
       <c r="A13" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="37" t="s">
-        <v>36</v>
-      </c>
       <c r="C13" s="37" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="F13" s="53" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="G13" s="37" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="H13" s="37" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="58" customHeight="1">
       <c r="A14" s="40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="F14" s="53" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="58" customHeight="1">
       <c r="A15" s="40" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="F15" s="53" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="H15" s="37" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="58" customHeight="1">
       <c r="A16" s="40" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F16" s="53" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="58" customHeight="1">
       <c r="A17" s="40" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C17" s="37" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="F17" s="53" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="G17" s="37" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H17" s="37" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="58" customHeight="1">
       <c r="A18" s="40" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C18" s="37" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="F18" s="53" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="58" customHeight="1">
       <c r="A19" s="40" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="D19" s="37" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="F19" s="53" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="G19" s="37" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="H19" s="37" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="58" customHeight="1">
       <c r="A20" s="40" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="F20" s="53" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="G20" s="37" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="H20" s="37" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="58" customHeight="1">
       <c r="A21" s="40" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F21" s="53" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="G21" s="37" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="72" customHeight="1">
@@ -5130,107 +5350,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="28" customHeight="1">
-      <c r="A1" s="66" t="s">
-        <v>245</v>
-      </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
+      <c r="A1" s="70" t="s">
+        <v>238</v>
+      </c>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
     </row>
     <row r="3" spans="1:16" ht="14.5">
-      <c r="A3" s="67" t="s">
-        <v>246</v>
-      </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
+      <c r="A3" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" s="71"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71"/>
+      <c r="P3" s="71"/>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="H5" s="17" t="s">
         <v>247</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="I5" s="17" t="s">
         <v>248</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="J5" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="K5" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="L5" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="M5" s="17" t="s">
         <v>252</v>
       </c>
-      <c r="G5" s="17" t="s">
+      <c r="N5" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="O5" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="P5" s="17" t="s">
         <v>255</v>
-      </c>
-      <c r="J5" s="17" t="s">
-        <v>256</v>
-      </c>
-      <c r="K5" s="17" t="s">
-        <v>257</v>
-      </c>
-      <c r="L5" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="M5" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="N5" s="17" t="s">
-        <v>260</v>
-      </c>
-      <c r="O5" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="P5" s="17" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="48" customHeight="1">
       <c r="A6" s="12" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E6" s="12">
         <v>366</v>
@@ -5251,36 +5471,36 @@
         <v>135.816</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="L6" s="14">
         <v>214883</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="O6" s="18" t="s">
         <v>7</v>
       </c>
       <c r="P6" s="12" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="48" customHeight="1">
       <c r="A7" s="12" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E7" s="12">
         <v>448</v>
@@ -5301,36 +5521,36 @@
         <v>230.15</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="L7" s="14">
         <v>0</v>
       </c>
       <c r="M7" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="O7" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="P7" s="12" t="s">
         <v>268</v>
-      </c>
-      <c r="O7" s="19" t="s">
-        <v>274</v>
-      </c>
-      <c r="P7" s="12" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="48" customHeight="1">
       <c r="A8" s="12" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="E8" s="12">
         <v>494</v>
@@ -5347,36 +5567,36 @@
         <v>100</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="L8" s="14">
         <v>39965</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="48" customHeight="1">
       <c r="A9" s="12" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E9" s="12">
         <v>508</v>
@@ -5397,36 +5617,36 @@
         <v>100.002</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="L9" s="14">
         <v>0</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="O9" s="19" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="P9" s="12" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="48" customHeight="1">
       <c r="A10" s="12" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E10" s="12">
         <v>4551</v>
@@ -5447,302 +5667,302 @@
         <v>100</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="L10" s="14">
         <v>0</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="O10" s="19" t="s">
         <v>5</v>
       </c>
       <c r="P10" s="12" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="68" t="s">
-        <v>295</v>
-      </c>
-      <c r="B11" s="68"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="68"/>
-      <c r="E11" s="68"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="68"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="68"/>
-      <c r="L11" s="68"/>
-      <c r="M11" s="68"/>
-      <c r="N11" s="68"/>
-      <c r="O11" s="68"/>
-      <c r="P11" s="68"/>
+      <c r="A11" s="72" t="s">
+        <v>288</v>
+      </c>
+      <c r="B11" s="72"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="72"/>
+      <c r="F11" s="72"/>
+      <c r="G11" s="72"/>
+      <c r="H11" s="72"/>
+      <c r="I11" s="72"/>
+      <c r="J11" s="72"/>
+      <c r="K11" s="72"/>
+      <c r="L11" s="72"/>
+      <c r="M11" s="72"/>
+      <c r="N11" s="72"/>
+      <c r="O11" s="72"/>
+      <c r="P11" s="72"/>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="21" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" s="15" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="15" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="15" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="17" spans="1:16">
-      <c r="A17" s="68" t="s">
-        <v>307</v>
-      </c>
-      <c r="B17" s="68"/>
-      <c r="C17" s="68"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="68"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="68"/>
-      <c r="M17" s="68"/>
-      <c r="N17" s="68"/>
-      <c r="O17" s="68"/>
-      <c r="P17" s="68"/>
+      <c r="A17" s="72" t="s">
+        <v>300</v>
+      </c>
+      <c r="B17" s="72"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="72"/>
+      <c r="E17" s="72"/>
+      <c r="F17" s="72"/>
+      <c r="G17" s="72"/>
+      <c r="H17" s="72"/>
+      <c r="I17" s="72"/>
+      <c r="J17" s="72"/>
+      <c r="K17" s="72"/>
+      <c r="L17" s="72"/>
+      <c r="M17" s="72"/>
+      <c r="N17" s="72"/>
+      <c r="O17" s="72"/>
+      <c r="P17" s="72"/>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" s="21" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
     </row>
     <row r="19" spans="1:16">
       <c r="A19" s="15" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="B19" s="15">
         <v>12.465999999999999</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="E19" s="16">
         <v>-1.2466E-2</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" spans="1:16">
       <c r="A20" s="15" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="B20" s="15">
         <v>-11.734</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="E20" s="16">
         <v>1.1734E-2</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="21" spans="1:16">
       <c r="A21" s="15" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="B21" s="15">
         <v>11.331</v>
       </c>
       <c r="C21" s="15" t="s">
+        <v>307</v>
+      </c>
+      <c r="D21" s="15" t="s">
         <v>314</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>321</v>
       </c>
       <c r="E21" s="16">
         <v>-1.1331000000000001E-2</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="15" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="B22" s="15">
         <v>29.593</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="E22" s="16">
         <v>-2.9593000000000001E-2</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="24" spans="1:16">
-      <c r="A24" s="68" t="s">
-        <v>324</v>
-      </c>
-      <c r="B24" s="68"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="68"/>
-      <c r="L24" s="68"/>
-      <c r="M24" s="68"/>
-      <c r="N24" s="68"/>
-      <c r="O24" s="68"/>
-      <c r="P24" s="68"/>
+      <c r="A24" s="72" t="s">
+        <v>317</v>
+      </c>
+      <c r="B24" s="72"/>
+      <c r="C24" s="72"/>
+      <c r="D24" s="72"/>
+      <c r="E24" s="72"/>
+      <c r="F24" s="72"/>
+      <c r="G24" s="72"/>
+      <c r="H24" s="72"/>
+      <c r="I24" s="72"/>
+      <c r="J24" s="72"/>
+      <c r="K24" s="72"/>
+      <c r="L24" s="72"/>
+      <c r="M24" s="72"/>
+      <c r="N24" s="72"/>
+      <c r="O24" s="72"/>
+      <c r="P24" s="72"/>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="H25" s="17" t="s">
         <v>247</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="I25" s="17" t="s">
         <v>248</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="J25" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="K25" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="L25" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="M25" s="17" t="s">
         <v>252</v>
       </c>
-      <c r="G25" s="17" t="s">
+      <c r="N25" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="H25" s="17" t="s">
+      <c r="O25" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="I25" s="17" t="s">
+      <c r="P25" s="17" t="s">
         <v>255</v>
-      </c>
-      <c r="J25" s="17" t="s">
-        <v>256</v>
-      </c>
-      <c r="K25" s="17" t="s">
-        <v>257</v>
-      </c>
-      <c r="L25" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="M25" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="N25" s="17" t="s">
-        <v>260</v>
-      </c>
-      <c r="O25" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="P25" s="17" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="52" customHeight="1">
       <c r="A26" s="12" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E26" s="12">
         <v>16621</v>
@@ -5763,106 +5983,106 @@
         <v>99.998999999999995</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="L26" s="14">
         <v>0</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="N26" s="12" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="O26" s="19" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="P26" s="12" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
     </row>
     <row r="28" spans="1:16">
-      <c r="A28" s="68" t="s">
-        <v>331</v>
-      </c>
-      <c r="B28" s="68"/>
-      <c r="C28" s="68"/>
-      <c r="D28" s="68"/>
-      <c r="E28" s="68"/>
-      <c r="F28" s="68"/>
-      <c r="G28" s="68"/>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="68"/>
-      <c r="K28" s="68"/>
-      <c r="L28" s="68"/>
-      <c r="M28" s="68"/>
-      <c r="N28" s="68"/>
-      <c r="O28" s="68"/>
-      <c r="P28" s="68"/>
+      <c r="A28" s="72" t="s">
+        <v>324</v>
+      </c>
+      <c r="B28" s="72"/>
+      <c r="C28" s="72"/>
+      <c r="D28" s="72"/>
+      <c r="E28" s="72"/>
+      <c r="F28" s="72"/>
+      <c r="G28" s="72"/>
+      <c r="H28" s="72"/>
+      <c r="I28" s="72"/>
+      <c r="J28" s="72"/>
+      <c r="K28" s="72"/>
+      <c r="L28" s="72"/>
+      <c r="M28" s="72"/>
+      <c r="N28" s="72"/>
+      <c r="O28" s="72"/>
+      <c r="P28" s="72"/>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="H29" s="17" t="s">
         <v>247</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="I29" s="17" t="s">
         <v>248</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="J29" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="K29" s="17" t="s">
         <v>250</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="L29" s="17" t="s">
         <v>251</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="M29" s="17" t="s">
         <v>252</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="N29" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="H29" s="17" t="s">
+      <c r="O29" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="I29" s="17" t="s">
+      <c r="P29" s="17" t="s">
         <v>255</v>
-      </c>
-      <c r="J29" s="17" t="s">
-        <v>256</v>
-      </c>
-      <c r="K29" s="17" t="s">
-        <v>257</v>
-      </c>
-      <c r="L29" s="17" t="s">
-        <v>258</v>
-      </c>
-      <c r="M29" s="17" t="s">
-        <v>259</v>
-      </c>
-      <c r="N29" s="17" t="s">
-        <v>260</v>
-      </c>
-      <c r="O29" s="17" t="s">
-        <v>261</v>
-      </c>
-      <c r="P29" s="17" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="48" customHeight="1">
       <c r="A30" s="12" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E30" s="12">
         <v>3135</v>
@@ -5883,82 +6103,82 @@
         <v>100</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="L30" s="14">
         <v>0</v>
       </c>
       <c r="M30" s="12" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="N30" s="12" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="O30" s="19" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="P30" s="12" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
     </row>
     <row r="32" spans="1:16">
-      <c r="A32" s="68" t="s">
-        <v>338</v>
-      </c>
-      <c r="B32" s="68"/>
-      <c r="C32" s="68"/>
-      <c r="D32" s="68"/>
-      <c r="E32" s="68"/>
-      <c r="F32" s="68"/>
-      <c r="G32" s="68"/>
-      <c r="H32" s="68"/>
-      <c r="I32" s="68"/>
-      <c r="J32" s="68"/>
-      <c r="K32" s="68"/>
-      <c r="L32" s="68"/>
-      <c r="M32" s="68"/>
-      <c r="N32" s="68"/>
-      <c r="O32" s="68"/>
-      <c r="P32" s="68"/>
+      <c r="A32" s="72" t="s">
+        <v>331</v>
+      </c>
+      <c r="B32" s="72"/>
+      <c r="C32" s="72"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="72"/>
+      <c r="G32" s="72"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="72"/>
+      <c r="J32" s="72"/>
+      <c r="K32" s="72"/>
+      <c r="L32" s="72"/>
+      <c r="M32" s="72"/>
+      <c r="N32" s="72"/>
+      <c r="O32" s="72"/>
+      <c r="P32" s="72"/>
     </row>
     <row r="33" spans="1:16" ht="32" customHeight="1">
       <c r="A33" s="33" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="E33" s="33" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="F33" s="33" t="s">
-        <v>344</v>
-      </c>
-      <c r="G33" s="69" t="s">
-        <v>345</v>
-      </c>
-      <c r="H33" s="69"/>
-      <c r="I33" s="69"/>
-      <c r="J33" s="69"/>
-      <c r="K33" s="69"/>
-      <c r="L33" s="69"/>
-      <c r="M33" s="69"/>
-      <c r="N33" s="69"/>
-      <c r="O33" s="69"/>
-      <c r="P33" s="69"/>
+        <v>337</v>
+      </c>
+      <c r="G33" s="74" t="s">
+        <v>338</v>
+      </c>
+      <c r="H33" s="74"/>
+      <c r="I33" s="74"/>
+      <c r="J33" s="74"/>
+      <c r="K33" s="74"/>
+      <c r="L33" s="74"/>
+      <c r="M33" s="74"/>
+      <c r="N33" s="74"/>
+      <c r="O33" s="74"/>
+      <c r="P33" s="74"/>
     </row>
     <row r="34" spans="1:16" ht="46" customHeight="1">
       <c r="A34" s="39" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="C34" s="54">
         <v>41</v>
@@ -5970,27 +6190,27 @@
         <v>26.9</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>348</v>
-      </c>
-      <c r="G34" s="70" t="s">
-        <v>349</v>
-      </c>
-      <c r="H34" s="70"/>
-      <c r="I34" s="70"/>
-      <c r="J34" s="70"/>
-      <c r="K34" s="70"/>
-      <c r="L34" s="70"/>
-      <c r="M34" s="70"/>
-      <c r="N34" s="70"/>
-      <c r="O34" s="70"/>
-      <c r="P34" s="70"/>
+        <v>341</v>
+      </c>
+      <c r="G34" s="73" t="s">
+        <v>342</v>
+      </c>
+      <c r="H34" s="73"/>
+      <c r="I34" s="73"/>
+      <c r="J34" s="73"/>
+      <c r="K34" s="73"/>
+      <c r="L34" s="73"/>
+      <c r="M34" s="73"/>
+      <c r="N34" s="73"/>
+      <c r="O34" s="73"/>
+      <c r="P34" s="73"/>
     </row>
     <row r="35" spans="1:16" ht="46" customHeight="1">
       <c r="A35" s="39" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="C35" s="54">
         <v>42.9</v>
@@ -6002,27 +6222,27 @@
         <v>28.6</v>
       </c>
       <c r="F35" s="37" t="s">
-        <v>348</v>
-      </c>
-      <c r="G35" s="70" t="s">
-        <v>351</v>
-      </c>
-      <c r="H35" s="70"/>
-      <c r="I35" s="70"/>
-      <c r="J35" s="70"/>
-      <c r="K35" s="70"/>
-      <c r="L35" s="70"/>
-      <c r="M35" s="70"/>
-      <c r="N35" s="70"/>
-      <c r="O35" s="70"/>
-      <c r="P35" s="70"/>
+        <v>341</v>
+      </c>
+      <c r="G35" s="73" t="s">
+        <v>344</v>
+      </c>
+      <c r="H35" s="73"/>
+      <c r="I35" s="73"/>
+      <c r="J35" s="73"/>
+      <c r="K35" s="73"/>
+      <c r="L35" s="73"/>
+      <c r="M35" s="73"/>
+      <c r="N35" s="73"/>
+      <c r="O35" s="73"/>
+      <c r="P35" s="73"/>
     </row>
     <row r="36" spans="1:16" ht="46" customHeight="1">
       <c r="A36" s="39" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="C36" s="54">
         <v>42.9</v>
@@ -6034,20 +6254,20 @@
         <v>27.6</v>
       </c>
       <c r="F36" s="37" t="s">
-        <v>348</v>
-      </c>
-      <c r="G36" s="70" t="s">
-        <v>353</v>
-      </c>
-      <c r="H36" s="70"/>
-      <c r="I36" s="70"/>
-      <c r="J36" s="70"/>
-      <c r="K36" s="70"/>
-      <c r="L36" s="70"/>
-      <c r="M36" s="70"/>
-      <c r="N36" s="70"/>
-      <c r="O36" s="70"/>
-      <c r="P36" s="70"/>
+        <v>341</v>
+      </c>
+      <c r="G36" s="73" t="s">
+        <v>346</v>
+      </c>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="73"/>
+      <c r="M36" s="73"/>
+      <c r="N36" s="73"/>
+      <c r="O36" s="73"/>
+      <c r="P36" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>